<commit_message>
started adding primers for invertebrates
</commit_message>
<xml_diff>
--- a/Project_clone/Report/primer_data.xlsx
+++ b/Project_clone/Report/primer_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="65">
   <si>
     <t xml:space="preserve">Typ av analys</t>
   </si>
@@ -136,7 +136,7 @@
     <t xml:space="preserve">55-50</t>
   </si>
   <si>
-    <t xml:space="preserve">Insekter</t>
+    <t xml:space="preserve">Insekter (COI)</t>
   </si>
   <si>
     <t xml:space="preserve">CCHGAYATRGCHTTYCCHCG</t>
@@ -145,6 +145,9 @@
     <t xml:space="preserve">TCDGGRTGNCCRAARAAYCA</t>
   </si>
   <si>
+    <t xml:space="preserve">IBA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nitella\_meta</t>
   </si>
   <si>
@@ -209,6 +212,9 @@
   </si>
   <si>
     <t xml:space="preserve">Valentini et al. 2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EPT</t>
   </si>
 </sst>
 </file>
@@ -289,7 +295,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -300,10 +306,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -437,7 +439,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.27"/>
@@ -526,7 +528,7 @@
       <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -568,10 +570,10 @@
       <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -614,16 +616,19 @@
       <c r="E9" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="F9" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>10</v>
@@ -634,7 +639,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>18</v>
@@ -651,13 +656,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>10</v>
@@ -665,65 +670,76 @@
       <c r="E12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>48</v>
+      <c r="G12" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>51</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B14" s="4" t="s">
         <v>54</v>
       </c>
+      <c r="B14" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="C14" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>60</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>61</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>61</v>
+      <c r="F15" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added primer details for invertebrates
</commit_message>
<xml_diff>
--- a/Project_clone/Report/primer_data.xlsx
+++ b/Project_clone/Report/primer_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="69">
   <si>
     <t xml:space="preserve">Typ av analys</t>
   </si>
@@ -148,6 +148,9 @@
     <t xml:space="preserve">IBA</t>
   </si>
   <si>
+    <t xml:space="preserve">Elbrecht et al. 2019</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nitella\_meta</t>
   </si>
   <si>
@@ -214,7 +217,16 @@
     <t xml:space="preserve">Valentini et al. 2016</t>
   </si>
   <si>
+    <t xml:space="preserve">GGDACWGGWTGAACWGTWTAYCCHCC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAAACAAATARDGGTATTCGDTY</t>
+  </si>
+  <si>
     <t xml:space="preserve">EPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vamos et al. 2017</t>
   </si>
 </sst>
 </file>
@@ -619,16 +631,19 @@
       <c r="F9" s="1" t="s">
         <v>41</v>
       </c>
+      <c r="G9" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>10</v>
@@ -639,7 +654,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>18</v>
@@ -656,13 +671,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>10</v>
@@ -671,75 +686,96 @@
         <v>20</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>55</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="B16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="E16" s="1" t="s">
         <v>37</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>